<commit_message>
Modified product list datasets
</commit_message>
<xml_diff>
--- a/data/product_scoring/product_list_1_dev_07-01-2026.xlsx
+++ b/data/product_scoring/product_list_1_dev_07-01-2026.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -44,6 +44,12 @@
   </si>
   <si>
     <t xml:space="preserve">advertising_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">packaging_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">payment_fees</t>
   </si>
   <si>
     <t xml:space="preserve">number_of_orders</t>
@@ -402,7 +408,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AG16"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.77"/>
@@ -410,23 +416,23 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="16.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="26.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="20.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="28.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="15.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="13.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="12.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="25.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="22.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="15.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="17.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="16.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="14.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="16.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="1" width="16.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="24.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="20.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="28.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="15.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="13.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="25.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="22.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="15.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="17.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="16.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="14.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="16.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -523,16 +529,22 @@
       <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="AF1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="27.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>8.49</v>
@@ -549,74 +561,80 @@
       <c r="H2" s="2" t="n">
         <v>0.6792</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I2" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K2" s="3" t="n">
         <v>495000</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="L2" s="2" t="n">
         <v>0.0217</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="M2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>130900</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="O2" s="2" t="n">
         <v>700</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="P2" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O2" s="2" t="n">
+      <c r="Q2" s="2" t="n">
         <v>4.07513333333333</v>
       </c>
-      <c r="P2" s="2" t="n">
+      <c r="R2" s="2" t="n">
         <v>8.49</v>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="S2" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="R2" s="2" t="n">
+      <c r="T2" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="S2" s="2" t="n">
+      <c r="U2" s="2" t="n">
         <v>250000</v>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="V2" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="U2" s="2" t="n">
+      <c r="W2" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="X2" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="Y2" s="2" t="n">
         <v>34554</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="Z2" s="2" t="n">
         <v>268400</v>
       </c>
-      <c r="Y2" s="4" t="n">
+      <c r="AA2" s="4" t="n">
         <f aca="false">7700000+28600000</f>
         <v>36300000</v>
       </c>
-      <c r="Z2" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA2" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB2" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC2" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD2" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE2" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD2" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE2" s="2" t="n">
+      <c r="AF2" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG2" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -625,10 +643,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>9.594</v>
@@ -646,72 +664,78 @@
         <v>0.76752</v>
       </c>
       <c r="I3" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="K3" s="2" t="n">
         <v>1964</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>0.0143</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="M3" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>1604</v>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="O3" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="P3" s="2" t="n">
         <v>4.86</v>
       </c>
-      <c r="O3" s="2" t="n">
+      <c r="Q3" s="2" t="n">
         <v>6.16708</v>
       </c>
-      <c r="P3" s="2" t="n">
+      <c r="R3" s="2" t="n">
         <v>9.594</v>
       </c>
-      <c r="Q3" s="2" t="n">
+      <c r="S3" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="R3" s="2" t="n">
+      <c r="T3" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="S3" s="2" t="n">
+      <c r="U3" s="2" t="n">
         <v>93.6</v>
       </c>
-      <c r="T3" s="2" t="n">
+      <c r="V3" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="U3" s="2" t="n">
+      <c r="W3" s="2" t="n">
         <v>5040</v>
       </c>
-      <c r="V3" s="2" t="n">
+      <c r="X3" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W3" s="2" t="n">
+      <c r="Y3" s="2" t="n">
         <v>578974</v>
       </c>
-      <c r="X3" s="2" t="n">
+      <c r="Z3" s="2" t="n">
         <v>7780</v>
       </c>
-      <c r="Y3" s="4" t="n">
+      <c r="AA3" s="4" t="n">
         <v>17600000</v>
       </c>
-      <c r="Z3" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA3" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB3" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC3" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD3" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE3" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD3" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE3" s="2" t="n">
+      <c r="AF3" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG3" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -720,10 +744,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>6.536</v>
@@ -741,72 +765,78 @@
         <v>0.52288</v>
       </c>
       <c r="I4" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K4" s="2" t="n">
         <v>1646000</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>0.0315</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="M4" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>130200</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="O4" s="2" t="n">
         <v>360</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="P4" s="2" t="n">
         <v>4.94</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="Q4" s="2" t="n">
         <v>4.05952</v>
       </c>
-      <c r="P4" s="2" t="n">
+      <c r="R4" s="2" t="n">
         <v>6.536</v>
       </c>
-      <c r="Q4" s="2" t="n">
+      <c r="S4" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="R4" s="2" t="n">
+      <c r="T4" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="S4" s="2" t="n">
+      <c r="U4" s="2" t="n">
         <v>63.375</v>
       </c>
-      <c r="T4" s="2" t="n">
+      <c r="V4" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="U4" s="2" t="n">
+      <c r="W4" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="V4" s="2" t="n">
+      <c r="X4" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="W4" s="2" t="n">
+      <c r="Y4" s="2" t="n">
         <v>2152690</v>
       </c>
-      <c r="X4" s="2" t="n">
+      <c r="Z4" s="2" t="n">
         <v>73000</v>
       </c>
-      <c r="Y4" s="4" t="n">
+      <c r="AA4" s="4" t="n">
         <v>690800000</v>
       </c>
-      <c r="Z4" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA4" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB4" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC4" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD4" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE4" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD4" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE4" s="2" t="n">
+      <c r="AF4" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG4" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -815,10 +845,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>11.76</v>
@@ -836,72 +866,78 @@
         <v>0.9408</v>
       </c>
       <c r="I5" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>13069</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="L5" s="2" t="n">
         <v>0.0315</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="M5" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="N5" s="2" t="n">
         <v>3046</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="O5" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="P5" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="Q5" s="2" t="n">
         <v>6.1257</v>
       </c>
-      <c r="P5" s="2" t="n">
+      <c r="R5" s="2" t="n">
         <v>11.76</v>
       </c>
-      <c r="Q5" s="2" t="n">
+      <c r="S5" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="R5" s="2" t="n">
+      <c r="T5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S5" s="2" t="n">
+      <c r="U5" s="2" t="n">
         <v>7.314</v>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="V5" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="U5" s="2" t="n">
+      <c r="W5" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="X5" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W5" s="2" t="n">
+      <c r="Y5" s="2" t="n">
         <v>746493</v>
       </c>
-      <c r="X5" s="2" t="n">
+      <c r="Z5" s="2" t="n">
         <v>1232</v>
       </c>
-      <c r="Y5" s="4" t="n">
+      <c r="AA5" s="4" t="n">
         <v>17600000</v>
       </c>
-      <c r="Z5" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA5" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB5" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC5" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD5" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE5" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD5" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE5" s="2" t="n">
+      <c r="AF5" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG5" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -910,10 +946,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>28.8011111111111</v>
@@ -931,72 +967,78 @@
         <v>2.30408888888889</v>
       </c>
       <c r="I6" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K6" s="2" t="n">
         <v>152028</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="L6" s="2" t="n">
         <v>0.0161</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="M6" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>17142</v>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="O6" s="2" t="n">
         <v>840</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="P6" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="Q6" s="2" t="n">
         <v>23.8418</v>
       </c>
-      <c r="P6" s="2" t="n">
+      <c r="R6" s="2" t="n">
         <v>28.8</v>
       </c>
-      <c r="Q6" s="2" t="n">
+      <c r="S6" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="R6" s="2" t="n">
+      <c r="T6" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="S6" s="2" t="n">
+      <c r="U6" s="2" t="n">
         <v>2268</v>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="V6" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="U6" s="2" t="n">
+      <c r="W6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V6" s="2" t="n">
+      <c r="X6" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W6" s="2" t="n">
+      <c r="Y6" s="2" t="n">
         <v>1449788</v>
       </c>
-      <c r="X6" s="2" t="n">
+      <c r="Z6" s="2" t="n">
         <v>203200</v>
       </c>
-      <c r="Y6" s="4" t="n">
+      <c r="AA6" s="4" t="n">
         <v>1100000000</v>
       </c>
-      <c r="Z6" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA6" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB6" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC6" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD6" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE6" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD6" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE6" s="2" t="n">
+      <c r="AF6" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG6" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1005,10 +1047,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>7.12</v>
@@ -1026,72 +1068,78 @@
         <v>0.5696</v>
       </c>
       <c r="I7" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K7" s="2" t="n">
         <v>819000</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="L7" s="2" t="n">
         <v>0.0236</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="M7" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="N7" s="2" t="n">
         <v>95893</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="O7" s="2" t="n">
         <v>900</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="P7" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="Q7" s="2" t="n">
         <v>4.2744</v>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="R7" s="2" t="n">
         <v>7.12</v>
       </c>
-      <c r="Q7" s="2" t="n">
+      <c r="S7" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="R7" s="2" t="n">
+      <c r="T7" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="S7" s="2" t="n">
+      <c r="U7" s="2" t="n">
         <v>275</v>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="V7" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="U7" s="2" t="n">
+      <c r="W7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V7" s="2" t="n">
+      <c r="X7" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W7" s="2" t="n">
+      <c r="Y7" s="2" t="n">
         <v>194243</v>
       </c>
-      <c r="X7" s="2" t="n">
+      <c r="Z7" s="2" t="n">
         <v>23100</v>
       </c>
-      <c r="Y7" s="4" t="n">
+      <c r="AA7" s="4" t="n">
         <v>9200000</v>
       </c>
-      <c r="Z7" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA7" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB7" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC7" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD7" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE7" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD7" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE7" s="2" t="n">
+      <c r="AF7" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG7" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1100,10 +1148,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>17.418</v>
@@ -1121,72 +1169,78 @@
         <v>1.39344</v>
       </c>
       <c r="I8" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K8" s="2" t="n">
         <v>4407</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="L8" s="2" t="n">
         <v>0.0315</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="M8" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>1611</v>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="O8" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="P8" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="Q8" s="2" t="n">
         <v>10.93076</v>
       </c>
-      <c r="P8" s="2" t="n">
+      <c r="R8" s="2" t="n">
         <v>17.418</v>
       </c>
-      <c r="Q8" s="2" t="n">
+      <c r="S8" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="R8" s="2" t="n">
+      <c r="T8" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="S8" s="2" t="n">
+      <c r="U8" s="2" t="n">
         <v>127.5</v>
       </c>
-      <c r="T8" s="2" t="n">
+      <c r="V8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="U8" s="2" t="n">
+      <c r="W8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V8" s="2" t="n">
+      <c r="X8" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W8" s="2" t="n">
+      <c r="Y8" s="2" t="n">
         <v>5509800</v>
       </c>
-      <c r="X8" s="2" t="n">
+      <c r="Z8" s="2" t="n">
         <v>76100</v>
       </c>
-      <c r="Y8" s="4" t="n">
+      <c r="AA8" s="4" t="n">
         <v>192800000</v>
       </c>
-      <c r="Z8" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA8" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB8" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC8" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD8" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE8" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD8" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE8" s="2" t="n">
+      <c r="AF8" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG8" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1195,10 +1249,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>11.298</v>
@@ -1216,72 +1270,78 @@
         <v>0.90384</v>
       </c>
       <c r="I9" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K9" s="2" t="n">
         <v>1282000</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>0.0315</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="M9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>230742</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="O9" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="P9" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O9" s="2" t="n">
+      <c r="Q9" s="2" t="n">
         <v>5.66436</v>
       </c>
-      <c r="P9" s="2" t="n">
+      <c r="R9" s="2" t="n">
         <v>11.298</v>
       </c>
-      <c r="Q9" s="2" t="n">
+      <c r="S9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="R9" s="2" t="n">
+      <c r="T9" s="2" t="n">
         <v>187</v>
       </c>
-      <c r="S9" s="2" t="n">
+      <c r="U9" s="2" t="n">
         <v>212.96</v>
       </c>
-      <c r="T9" s="2" t="n">
+      <c r="V9" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="U9" s="2" t="n">
+      <c r="W9" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="V9" s="2" t="n">
+      <c r="X9" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W9" s="2" t="n">
+      <c r="Y9" s="2" t="n">
         <v>559364</v>
       </c>
-      <c r="X9" s="2" t="n">
+      <c r="Z9" s="2" t="n">
         <v>15200</v>
       </c>
-      <c r="Y9" s="2" t="n">
+      <c r="AA9" s="2" t="n">
         <v>301700000</v>
       </c>
-      <c r="Z9" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA9" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB9" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC9" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD9" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE9" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD9" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE9" s="2" t="n">
+      <c r="AF9" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG9" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1290,10 +1350,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>13.562</v>
@@ -1311,72 +1371,78 @@
         <v>1.08496</v>
       </c>
       <c r="I10" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K10" s="2" t="n">
         <v>250000</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="L10" s="2" t="n">
         <v>0.0315</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="M10" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>35481</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="O10" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="P10" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O10" s="2" t="n">
+      <c r="Q10" s="2" t="n">
         <v>7.52084</v>
       </c>
-      <c r="P10" s="2" t="n">
+      <c r="R10" s="2" t="n">
         <v>13.562</v>
       </c>
-      <c r="Q10" s="2" t="n">
+      <c r="S10" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="R10" s="2" t="n">
+      <c r="T10" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="S10" s="2" t="n">
+      <c r="U10" s="2" t="n">
         <v>202.5</v>
       </c>
-      <c r="T10" s="2" t="n">
+      <c r="V10" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="U10" s="2" t="n">
+      <c r="W10" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="V10" s="2" t="n">
+      <c r="X10" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W10" s="2" t="n">
+      <c r="Y10" s="2" t="n">
         <v>12276</v>
       </c>
-      <c r="X10" s="2" t="n">
+      <c r="Z10" s="2" t="n">
         <v>21100</v>
       </c>
-      <c r="Y10" s="2" t="n">
+      <c r="AA10" s="2" t="n">
         <v>3100000000</v>
       </c>
-      <c r="Z10" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA10" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB10" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC10" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD10" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE10" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD10" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE10" s="2" t="n">
+      <c r="AF10" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG10" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1385,10 +1451,10 @@
         <v>12</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>12.12</v>
@@ -1406,72 +1472,78 @@
         <v>0.9696</v>
       </c>
       <c r="I11" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K11" s="2" t="n">
         <v>174910</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="L11" s="2" t="n">
         <v>0.0779</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="M11" s="2" t="n">
         <v>4.82142857142857</v>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>37945</v>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="O11" s="2" t="n">
         <v>720</v>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="P11" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="Q11" s="2" t="n">
         <v>6.9064</v>
       </c>
-      <c r="P11" s="2" t="n">
+      <c r="R11" s="2" t="n">
         <v>12.12</v>
       </c>
-      <c r="Q11" s="2" t="n">
+      <c r="S11" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="R11" s="2" t="n">
+      <c r="T11" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="S11" s="2" t="n">
+      <c r="U11" s="2" t="n">
         <v>3618</v>
       </c>
-      <c r="T11" s="2" t="n">
+      <c r="V11" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="U11" s="2" t="n">
+      <c r="W11" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="V11" s="2" t="n">
+      <c r="X11" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W11" s="2" t="n">
+      <c r="Y11" s="2" t="n">
         <v>549877</v>
       </c>
-      <c r="X11" s="2" t="n">
+      <c r="Z11" s="2" t="n">
         <v>5800</v>
       </c>
-      <c r="Y11" s="2" t="n">
+      <c r="AA11" s="2" t="n">
         <v>43593000</v>
       </c>
-      <c r="Z11" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA11" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB11" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC11" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD11" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE11" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD11" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE11" s="2" t="n">
+      <c r="AF11" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG11" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1480,10 +1552,10 @@
         <v>13</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>4.252</v>
@@ -1501,72 +1573,78 @@
         <v>0.34016</v>
       </c>
       <c r="I12" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="K12" s="2" t="n">
         <v>665152</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="L12" s="2" t="n">
         <v>0.0779</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="M12" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="N12" s="2" t="n">
         <v>87673</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="O12" s="2" t="n">
         <v>360</v>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="P12" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="O12" s="2" t="n">
+      <c r="Q12" s="2" t="n">
         <v>1.73864</v>
       </c>
-      <c r="P12" s="2" t="n">
+      <c r="R12" s="2" t="n">
         <v>4.252</v>
       </c>
-      <c r="Q12" s="2" t="n">
+      <c r="S12" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="R12" s="2" t="n">
+      <c r="T12" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="S12" s="2" t="n">
+      <c r="U12" s="2" t="n">
         <v>234.6</v>
       </c>
-      <c r="T12" s="2" t="n">
+      <c r="V12" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="U12" s="2" t="n">
+      <c r="W12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V12" s="2" t="n">
+      <c r="X12" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W12" s="2" t="n">
+      <c r="Y12" s="2" t="n">
         <v>2129700</v>
       </c>
-      <c r="X12" s="2" t="n">
+      <c r="Z12" s="2" t="n">
         <v>7600</v>
       </c>
-      <c r="Y12" s="2" t="n">
+      <c r="AA12" s="2" t="n">
         <v>95500000</v>
       </c>
-      <c r="Z12" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA12" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB12" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC12" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD12" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE12" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD12" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE12" s="2" t="n">
+      <c r="AF12" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG12" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1575,10 +1653,10 @@
         <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>9.442</v>
@@ -1596,72 +1674,78 @@
         <v>0.75536</v>
       </c>
       <c r="I13" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="K13" s="2" t="n">
         <v>32026</v>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="L13" s="2" t="n">
         <v>0.0161</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="M13" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L13" s="2" t="n">
+      <c r="N13" s="2" t="n">
         <v>10414</v>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="O13" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="P13" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="O13" s="2" t="n">
+      <c r="Q13" s="2" t="n">
         <v>5.14244</v>
       </c>
-      <c r="P13" s="2" t="n">
+      <c r="R13" s="2" t="n">
         <v>5.77084</v>
       </c>
-      <c r="Q13" s="2" t="n">
+      <c r="S13" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="R13" s="2" t="n">
+      <c r="T13" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="S13" s="2" t="n">
+      <c r="U13" s="2" t="n">
         <v>5850</v>
       </c>
-      <c r="T13" s="2" t="n">
+      <c r="V13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U13" s="2" t="n">
+      <c r="W13" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="V13" s="2" t="n">
+      <c r="X13" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="W13" s="2" t="n">
+      <c r="Y13" s="2" t="n">
         <v>662282</v>
       </c>
-      <c r="X13" s="2" t="n">
+      <c r="Z13" s="2" t="n">
         <v>222</v>
       </c>
-      <c r="Y13" s="2" t="n">
+      <c r="AA13" s="2" t="n">
         <v>2220000</v>
       </c>
-      <c r="Z13" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA13" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB13" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC13" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD13" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE13" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD13" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE13" s="2" t="n">
+      <c r="AF13" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG13" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1670,10 +1754,10 @@
         <v>15</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>6.128</v>
@@ -1691,72 +1775,78 @@
         <v>0.49024</v>
       </c>
       <c r="I14" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K14" s="2" t="n">
         <v>360466</v>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="L14" s="2" t="n">
         <v>0.0779</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="M14" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>40831</v>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="O14" s="2" t="n">
         <v>660</v>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="P14" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="O14" s="2" t="n">
+      <c r="Q14" s="2" t="n">
         <v>3.52496</v>
       </c>
-      <c r="P14" s="2" t="n">
+      <c r="R14" s="2" t="n">
         <v>6.128</v>
       </c>
-      <c r="Q14" s="2" t="n">
+      <c r="S14" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="R14" s="2" t="n">
+      <c r="T14" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="S14" s="2" t="n">
+      <c r="U14" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="T14" s="2" t="n">
+      <c r="V14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U14" s="2" t="n">
+      <c r="W14" s="2" t="n">
         <v>5000</v>
       </c>
-      <c r="V14" s="2" t="n">
+      <c r="X14" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="W14" s="2" t="n">
+      <c r="Y14" s="2" t="n">
         <v>1505900</v>
       </c>
-      <c r="X14" s="2" t="n">
+      <c r="Z14" s="2" t="n">
         <v>127300</v>
       </c>
-      <c r="Y14" s="2" t="n">
+      <c r="AA14" s="2" t="n">
         <v>7000000000</v>
       </c>
-      <c r="Z14" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA14" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB14" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC14" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD14" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE14" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD14" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE14" s="2" t="n">
+      <c r="AF14" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG14" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1765,10 +1855,10 @@
         <v>16</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>8.77</v>
@@ -1786,72 +1876,78 @@
         <v>0.7016</v>
       </c>
       <c r="I15" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="K15" s="2" t="n">
         <v>534141</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>0.0779</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="M15" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>51540</v>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="O15" s="2" t="n">
         <v>240</v>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="P15" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O15" s="2" t="n">
+      <c r="Q15" s="2" t="n">
         <v>4.4314</v>
       </c>
-      <c r="P15" s="2" t="n">
+      <c r="R15" s="2" t="n">
         <v>8.77</v>
       </c>
-      <c r="Q15" s="2" t="n">
+      <c r="S15" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="R15" s="2" t="n">
+      <c r="T15" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="S15" s="2" t="n">
+      <c r="U15" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="T15" s="2" t="n">
+      <c r="V15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U15" s="2" t="n">
+      <c r="W15" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="V15" s="2" t="n">
+      <c r="X15" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="W15" s="2" t="n">
+      <c r="Y15" s="2" t="n">
         <v>123421</v>
       </c>
-      <c r="X15" s="2" t="n">
+      <c r="Z15" s="2" t="n">
         <v>78000</v>
       </c>
-      <c r="Y15" s="2" t="n">
+      <c r="AA15" s="2" t="n">
         <v>716400000</v>
       </c>
-      <c r="Z15" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA15" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB15" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC15" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD15" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE15" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD15" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE15" s="2" t="n">
+      <c r="AF15" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG15" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1860,10 +1956,10 @@
         <v>17</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>9.848</v>
@@ -1881,72 +1977,78 @@
         <v>0.78784</v>
       </c>
       <c r="I16" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K16" s="2" t="n">
         <v>958500</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>0.0779</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="M16" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="N16" s="2" t="n">
         <v>78070</v>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="O16" s="2" t="n">
         <v>600</v>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="P16" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="O16" s="2" t="n">
+      <c r="Q16" s="2" t="n">
         <v>4.19336</v>
       </c>
-      <c r="P16" s="2" t="n">
+      <c r="R16" s="2" t="n">
         <v>9.848</v>
       </c>
-      <c r="Q16" s="2" t="n">
+      <c r="S16" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="R16" s="2" t="n">
+      <c r="T16" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="S16" s="2" t="n">
+      <c r="U16" s="2" t="n">
         <v>1188</v>
       </c>
-      <c r="T16" s="2" t="n">
+      <c r="V16" s="2" t="n">
         <v>4.9</v>
       </c>
-      <c r="U16" s="2" t="n">
+      <c r="W16" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="V16" s="2" t="n">
+      <c r="X16" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="W16" s="2" t="n">
+      <c r="Y16" s="2" t="n">
         <v>1547400</v>
       </c>
-      <c r="X16" s="2" t="n">
+      <c r="Z16" s="2" t="n">
         <v>4400</v>
       </c>
-      <c r="Y16" s="2" t="n">
+      <c r="AA16" s="2" t="n">
         <v>14890000</v>
       </c>
-      <c r="Z16" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA16" s="2" t="n">
-        <v>0.02</v>
-      </c>
       <c r="AB16" s="2" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AC16" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AD16" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AE16" s="2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AD16" s="2" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AE16" s="2" t="n">
+      <c r="AF16" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG16" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>

</xml_diff>